<commit_message>
Redetermine predicted mappings from the ontology's current synonyms
The DOID/SNOMED grounders read names and synonyms from the core report, a
master-list snapshot that still carried 148 synonyms withdrawn by the
synonym review and lacked 157 current ones. They now read the non-retired
diseases, live ARI_Synonym values and ARI_SNOMED codes from
ontologies/ari_t1d.owl via ari_diseases.py, as does report 8's Synonyms
column. Rerun the full pipeline and regenerate reports 5-8.

Top predictions now reproduce 649 of 713 curated mappings (was 641);
mismatches fall from 38 to 28.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/4-reports/5_DOID_Mapping.xlsx
+++ b/data/4-reports/5_DOID_Mapping.xlsx
@@ -740,17 +740,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.778</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>synonym</t>
+          <t>name</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>(preferred name)</t>
+          <t>autoimmune interstitial lung, joint, and kidney disease</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>

</xml_diff>